<commit_message>
Update disaster map Excel data
</commit_message>
<xml_diff>
--- a/data/재난현장지도_표준화_데이터.xlsx
+++ b/data/재난현장지도_표준화_데이터.xlsx
@@ -2897,14 +2897,14 @@
         <v>625</v>
       </c>
       <c r="H14" s="29">
-        <v>12000</v>
+        <v>12142</v>
       </c>
       <c r="I14" s="29">
         <v>18180</v>
       </c>
       <c r="J14" s="30">
         <f>SUM(B14:I14)</f>
-        <v>106057</v>
+        <v>106199</v>
       </c>
     </row>
     <row r="15" spans="1:10">

</xml_diff>